<commit_message>
Adiciona 4 lançamentos esquecidos e refinaliza a planilha
NOTE DE FRAIS HORS SEJOUR: lantica pizzeria Michèle repas guide (25€),
trenitalia Roma termini à l'aéroport (14€), etep opérations repas
guide (15,10€). FRAIS PIQUE-NIQUES: wine bar (36€). Recalcula
subtotais e TOTAL GÉNÉRAL (1.202,48€).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Notes de frais Pouilles du Sud 04-10-26.xlsx
+++ b/planilha/Notes de frais Pouilles du Sud 04-10-26.xlsx
@@ -533,7 +533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -664,228 +664,228 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>10/10/2026</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>lantica pizzeria Michèle repas guide</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>NOTE DE FRAIS HORS SEJOUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>10/10/2026</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>trenitalia Roma termini à l'aéroport</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>NOTE DE FRAIS HORS SEJOUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>10/10/2026</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>etep opérations repas guide</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>NOTE DE FRAIS HORS SEJOUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>Sous-total</t>
         </is>
       </c>
-      <c r="B7" s="8" t="n"/>
-      <c r="C7" s="8" t="n"/>
-      <c r="D7" s="9">
-        <f>SUM(D4:D6)</f>
+      <c r="B10" s="8" t="n"/>
+      <c r="C10" s="8" t="n"/>
+      <c r="D10" s="9">
+        <f>SUM(D4:D9)</f>
         <v/>
       </c>
-      <c r="E7" s="8" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="10" t="n"/>
-      <c r="B8" s="10" t="n"/>
-      <c r="C8" s="10" t="n"/>
-      <c r="D8" s="10" t="n"/>
-      <c r="E8" s="10" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="E10" s="8" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="n"/>
+      <c r="B11" s="10" t="n"/>
+      <c r="C11" s="10" t="n"/>
+      <c r="D11" s="10" t="n"/>
+      <c r="E11" s="10" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
         </is>
       </c>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="7" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="7" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>04/10/2026</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>train bari polignano+ ostuni-lecce</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="n">
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n">
         <v>136.5</v>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>04/10/2026</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>train Lecce Bari</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="n">
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="n">
         <v>178.5</v>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>04/10/2026</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>locorotondo-alberobello+ alberobello Martina+ Martina-cisternino</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="n">
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="n">
         <v>81</v>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>Sous-total</t>
         </is>
       </c>
-      <c r="B13" s="8" t="n"/>
-      <c r="C13" s="8" t="n"/>
-      <c r="D13" s="9">
-        <f>SUM(D10:D12)</f>
+      <c r="B16" s="8" t="n"/>
+      <c r="C16" s="8" t="n"/>
+      <c r="D16" s="9">
+        <f>SUM(D13:D15)</f>
         <v/>
       </c>
-      <c r="E13" s="8" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="10" t="n"/>
-      <c r="B14" s="10" t="n"/>
-      <c r="C14" s="10" t="n"/>
-      <c r="D14" s="10" t="n"/>
-      <c r="E14" s="10" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="E16" s="8" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="n"/>
+      <c r="B17" s="10" t="n"/>
+      <c r="C17" s="10" t="n"/>
+      <c r="D17" s="10" t="n"/>
+      <c r="E17" s="10" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>FRAIS PIQUE-NIQUES</t>
         </is>
       </c>
-      <c r="B15" s="6" t="n"/>
-      <c r="C15" s="6" t="n"/>
-      <c r="D15" s="6" t="n"/>
-      <c r="E15" s="7" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>04/10/2026</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>maiora</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="n">
-        <v>113.16</v>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>FRAIS PIQUE-NIQUES</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>05/10/2026</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>maiora</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="n">
-        <v>6.44</v>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>FRAIS PIQUE-NIQUES</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>05/10/2026</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>al vi erl Alberobello</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="n">
-        <v>57.1</v>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>FRAIS PIQUE-NIQUES</t>
-        </is>
-      </c>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="6" t="n"/>
+      <c r="D18" s="6" t="n"/>
+      <c r="E18" s="7" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
+          <t>04/10/2026</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>al vi erl Alberobello</t>
+          <t>maiora</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -894,7 +894,7 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>33.5</v>
+        <v>113.16</v>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
@@ -905,12 +905,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>05/10/2026</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>panificio</t>
+          <t>maiora</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -919,7 +919,7 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>8.949999999999999</v>
+        <v>6.44</v>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
@@ -930,12 +930,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>05/10/2026</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>macelleria</t>
+          <t>al vi erl Alberobello</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -944,7 +944,7 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>22</v>
+        <v>57.1</v>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
@@ -955,12 +955,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>06/10/2026</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Magic giov</t>
+          <t>al vi erl Alberobello</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -969,7 +969,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>120</v>
+        <v>33.5</v>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
@@ -980,12 +980,12 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>despar eurospar</t>
+          <t>panificio</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -994,7 +994,7 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>26.06</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
@@ -1005,12 +1005,12 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>wine bar (remplacement du repas à baia orte)</t>
+          <t>macelleria</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -1019,7 +1019,7 @@
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>214.5</v>
+        <v>22</v>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
@@ -1030,62 +1030,112 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Magic giov</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS PIQUE-NIQUES</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>despar eurospar</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>26.06</v>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS PIQUE-NIQUES</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
           <t>09/10/2026</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>wine bar (remplacement du repas à baia orte)</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>214.5</v>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS PIQUE-NIQUES</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>casamelia bakery</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="n">
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="n">
         <v>16.3</v>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>FRAIS PIQUE-NIQUES</t>
         </is>
       </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="8" t="inlineStr">
-        <is>
-          <t>Sous-total</t>
-        </is>
-      </c>
-      <c r="B26" s="8" t="n"/>
-      <c r="C26" s="8" t="n"/>
-      <c r="D26" s="9">
-        <f>SUM(D16:D25)</f>
-        <v/>
-      </c>
-      <c r="E26" s="8" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="5" t="inlineStr">
-        <is>
-          <t>FRAIS, TAXES DE SEJOUR, REPAS Accompagnateur</t>
-        </is>
-      </c>
-      <c r="B28" s="6" t="n"/>
-      <c r="C28" s="6" t="n"/>
-      <c r="D28" s="6" t="n"/>
-      <c r="E28" s="7" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>04/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>pizzeria Enzo e Ciro repas guide en séjour</t>
+          <t>wine bar</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -1094,11 +1144,11 @@
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>FRAIS, TAXES DE SEJOUR, REPAS Accompagnateur</t>
+          <t>FRAIS PIQUE-NIQUES</t>
         </is>
       </c>
     </row>
@@ -1111,15 +1161,22 @@
       <c r="B30" s="8" t="n"/>
       <c r="C30" s="8" t="n"/>
       <c r="D30" s="9">
-        <f>SUM(D29:D29)</f>
+        <f>SUM(D19:D29)</f>
         <v/>
       </c>
       <c r="E30" s="8" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="n"/>
+      <c r="B31" s="10" t="n"/>
+      <c r="C31" s="10" t="n"/>
+      <c r="D31" s="10" t="n"/>
+      <c r="E31" s="10" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>FRAIS VISITES</t>
+          <t>FRAIS, TAXES DE SEJOUR, REPAS Accompagnateur</t>
         </is>
       </c>
       <c r="B32" s="6" t="n"/>
@@ -1130,12 +1187,12 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>04/10/2026</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>mudo mosaïque otrante</t>
+          <t>pizzeria Enzo e Ciro repas guide en séjour</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -1144,11 +1201,11 @@
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>FRAIS VISITES</t>
+          <t>FRAIS, TAXES DE SEJOUR, REPAS Accompagnateur</t>
         </is>
       </c>
     </row>
@@ -1166,57 +1223,121 @@
       </c>
       <c r="E34" s="8" t="n"/>
     </row>
+    <row r="35">
+      <c r="A35" s="10" t="n"/>
+      <c r="B35" s="10" t="n"/>
+      <c r="C35" s="10" t="n"/>
+      <c r="D35" s="10" t="n"/>
+      <c r="E35" s="10" t="n"/>
+    </row>
     <row r="36">
-      <c r="A36" s="11" t="inlineStr">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>FRAIS VISITES</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="n"/>
+      <c r="C36" s="6" t="n"/>
+      <c r="D36" s="6" t="n"/>
+      <c r="E36" s="7" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>mudo mosaïque otrante</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS VISITES</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>Sous-total</t>
+        </is>
+      </c>
+      <c r="B38" s="8" t="n"/>
+      <c r="C38" s="8" t="n"/>
+      <c r="D38" s="9">
+        <f>SUM(D37:D37)</f>
+        <v/>
+      </c>
+      <c r="E38" s="8" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="10" t="n"/>
+      <c r="B39" s="10" t="n"/>
+      <c r="C39" s="10" t="n"/>
+      <c r="D39" s="10" t="n"/>
+      <c r="E39" s="10" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="11" t="inlineStr">
         <is>
           <t>TOTAL GÉNÉRAL</t>
         </is>
       </c>
-      <c r="B36" s="6" t="n"/>
-      <c r="C36" s="7" t="n"/>
-      <c r="D36" s="12">
-        <f>D7+D13+D26+D30+D34</f>
+      <c r="B40" s="6" t="n"/>
+      <c r="C40" s="7" t="n"/>
+      <c r="D40" s="12">
+        <f>D10+D16+D30+D34+D38</f>
         <v/>
       </c>
-      <c r="E36" s="11" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="13" t="inlineStr">
+      <c r="E40" s="11" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="13" t="inlineStr">
         <is>
           <t>Avance reçue</t>
         </is>
       </c>
-      <c r="B38" s="6" t="n"/>
-      <c r="C38" s="7" t="n"/>
-      <c r="D38" s="14" t="n">
-        <v>-0</v>
-      </c>
-      <c r="E38" s="13" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="11" t="inlineStr">
+      <c r="B42" s="6" t="n"/>
+      <c r="C42" s="7" t="n"/>
+      <c r="D42" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" s="13" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="11" t="inlineStr">
         <is>
           <t>MONTANT À REMBOURSER</t>
         </is>
       </c>
-      <c r="B39" s="6" t="n"/>
-      <c r="C39" s="7" t="n"/>
-      <c r="D39" s="15">
-        <f>D36+D38</f>
+      <c r="B43" s="6" t="n"/>
+      <c r="C43" s="7" t="n"/>
+      <c r="D43" s="15">
+        <f>D40+D42</f>
         <v/>
       </c>
-      <c r="E39" s="11" t="n"/>
+      <c r="E43" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="A36:C36"/>
-    <mergeCell ref="A15:E15"/>
-    <mergeCell ref="A28:E28"/>
-    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="A42:C42"/>
+    <mergeCell ref="A12:E12"/>
+    <mergeCell ref="A40:C40"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A32:E32"/>
-    <mergeCell ref="A39:C39"/>
-    <mergeCell ref="A9:E9"/>
+    <mergeCell ref="A36:E36"/>
+    <mergeCell ref="A43:C43"/>
+    <mergeCell ref="A18:E18"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>